<commit_message>
chore(security): remediate SCA vulnerabilities, add IDOR auth guards, and update reports
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/Security_Review_Report.xlsx
+++ b/Vulnerability Test Results/Security_Review_Report.xlsx
@@ -6,13 +6,14 @@
   <sheets>
     <sheet sheetId="1" name="Executive Summary" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Endpoint Inventory" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Findings Register" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="138">
   <si>
     <t>CODESAGA APPLICATION - SAST SECURITY &amp; DEVSECOPS AUDIT REPORT</t>
   </si>
@@ -26,7 +27,7 @@
     <t>Audit Date:</t>
   </si>
   <si>
-    <t>27/8/2026</t>
+    <t>26/10/2026</t>
   </si>
   <si>
     <t>Technology Stack:</t>
@@ -38,7 +39,7 @@
     <t>DevSecOps Tools:</t>
   </si>
   <si>
-    <t>Semgrep, Gitleaks, Trivy, Audit</t>
+    <t>Semgrep, Gitleaks, Trivy, npm audit</t>
   </si>
   <si>
     <t>Target Scope:</t>
@@ -47,52 +48,70 @@
     <t>Backend API, Authentication, Models, Routes</t>
   </si>
   <si>
-    <t>Overall Security Score:</t>
-  </si>
-  <si>
-    <t>A+ (98.5%)</t>
-  </si>
-  <si>
-    <t>🛡️ SECURITY AUDIT FINDINGS OVERVIEW</t>
-  </si>
-  <si>
-    <t>Finding Severity</t>
-  </si>
-  <si>
-    <t>Discovered Count</t>
-  </si>
-  <si>
-    <t>Remediated Count</t>
-  </si>
-  <si>
-    <t>Status Indicator</t>
-  </si>
-  <si>
-    <t>Critical Severity</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>CLEAN (0 Issues)</t>
-  </si>
-  <si>
-    <t>High Severity</t>
-  </si>
-  <si>
-    <t>Medium Severity</t>
-  </si>
-  <si>
-    <t>Low / Advisory Severity</t>
+    <t>Remediation Status:</t>
+  </si>
+  <si>
+    <t>Remediated &amp; Verified (20/20 Tests Passed)</t>
+  </si>
+  <si>
+    <t>🛡️ RECONCILED SECURITY FINDINGS &amp; REMEDIATION METRICS</t>
+  </si>
+  <si>
+    <t>Finding Category / Scope</t>
+  </si>
+  <si>
+    <t>Discovered</t>
+  </si>
+  <si>
+    <t>Remediated</t>
+  </si>
+  <si>
+    <t>Documented Pending</t>
+  </si>
+  <si>
+    <t>Verification Status</t>
+  </si>
+  <si>
+    <t>App Code — High (IDOR &amp; Rate Limiting)</t>
+  </si>
+  <si>
+    <t>REMEDIATED (Verified via Tests)</t>
+  </si>
+  <si>
+    <t>App Code — Medium (Headers &amp; Validation)</t>
+  </si>
+  <si>
+    <t>App Code — Low (PII Logging &amp; Error Leaks)</t>
+  </si>
+  <si>
+    <t>Dependencies (SCA) — Critical (proxy-addr, shell-quote)</t>
+  </si>
+  <si>
+    <t>REMEDIATED (0 Critical Remaining)</t>
+  </si>
+  <si>
+    <t>Dependencies (SCA) — High (Vite, body-parser, brace-expansion)</t>
+  </si>
+  <si>
+    <t>PARTIALLY REMEDIATED (5 in Expo CLI)</t>
+  </si>
+  <si>
+    <t>Dependencies (SCA) — Moderate (qs, query-string, uuid)</t>
+  </si>
+  <si>
+    <t>PARTIALLY REMEDIATED (2 in exceljs/uuid)</t>
   </si>
   <si>
     <t>Hardcoded Secrets (Gitleaks)</t>
   </si>
   <si>
-    <t>PASSED</t>
-  </si>
-  <si>
-    <t>Dependency Vulnerabilities (Trivy)</t>
+    <t>CLEAN (0 Secrets Detected)</t>
+  </si>
+  <si>
+    <t>Critical Security Gate Policy</t>
+  </si>
+  <si>
+    <t>PASSED (Zero Criticals)</t>
   </si>
   <si>
     <t>Endpoint Path</t>
@@ -128,7 +147,7 @@
     <t>server.js</t>
   </si>
   <si>
-    <t>Verified Safe</t>
+    <t>Verified Safe; Nosniff &amp; HSTS</t>
   </si>
   <si>
     <t>/</t>
@@ -137,7 +156,7 @@
     <t>/api/users/:email</t>
   </si>
   <si>
-    <t>Yes (Optional Guest)</t>
+    <t>Optional (Guest Allowed)</t>
   </si>
   <si>
     <t>User / Developer</t>
@@ -146,6 +165,9 @@
     <t>routes/users.js</t>
   </si>
   <si>
+    <t>Verified Safe; Email Normalization</t>
+  </si>
+  <si>
     <t>/api/users</t>
   </si>
   <si>
@@ -158,35 +180,260 @@
     <t>Public / User</t>
   </si>
   <si>
+    <t>Verified Safe; Password Complexity &amp; HMAC Token</t>
+  </si>
+  <si>
     <t>/api/users/set-password</t>
   </si>
   <si>
-    <t>Yes</t>
+    <t>Yes (Rate Limited)</t>
   </si>
   <si>
     <t>Verified User</t>
   </si>
   <si>
+    <t>Verified Safe; 10 req/15m Limit &amp; HMAC Token</t>
+  </si>
+  <si>
     <t>/api/users/login-password</t>
   </si>
   <si>
     <t>/api/users/login</t>
   </si>
   <si>
+    <t>Verified Safe; HMAC Token Issued</t>
+  </si>
+  <si>
     <t>/api/users/:email/progress</t>
   </si>
   <si>
+    <t>Yes (HMAC Bearer)</t>
+  </si>
+  <si>
+    <t>Own Account / Dev</t>
+  </si>
+  <si>
+    <t>Verified Safe; IDOR Ownership Protected</t>
+  </si>
+  <si>
     <t>PUT</t>
   </si>
   <si>
+    <t>Verified Safe; IDOR Protected &amp; Input Bounded</t>
+  </si>
+  <si>
     <t>/api/users/:email/certificate</t>
+  </si>
+  <si>
+    <t>Verified Safe; IDOR Protected &amp; World Validated</t>
+  </si>
+  <si>
+    <t>Finding ID</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Resource / Package</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Remediation Summary</t>
+  </si>
+  <si>
+    <t>SEC-01</t>
+  </si>
+  <si>
+    <t>App Code</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Auth &amp; Authorization</t>
+  </si>
+  <si>
+    <t>HMAC-SHA256 session token &amp; timing-safe ownership validation</t>
+  </si>
+  <si>
+    <t>SEC-02</t>
+  </si>
+  <si>
+    <t>Anti-Automation</t>
+  </si>
+  <si>
+    <t>Sliding-window IP rate limiter on login (10 attempts/15 min)</t>
+  </si>
+  <si>
+    <t>SEC-03</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Security Configuration</t>
+  </si>
+  <si>
+    <t>Defensive HTTP response headers (nosniff, SAMEORIGIN, HSTS, CSP)</t>
+  </si>
+  <si>
+    <t>SEC-04</t>
+  </si>
+  <si>
+    <t>Input Validation</t>
+  </si>
+  <si>
+    <t>validateProgressInput enforcing bounds on XP, level, coins, worlds</t>
+  </si>
+  <si>
+    <t>SEC-05</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Logging / PII</t>
+  </si>
+  <si>
+    <t>maskEmail helper masking plaintext emails in console output</t>
+  </si>
+  <si>
+    <t>SEC-06</t>
+  </si>
+  <si>
+    <t>Information Disclosure</t>
+  </si>
+  <si>
+    <t>server.js &amp; routes/users.js</t>
+  </si>
+  <si>
+    <t>safeErrorResponse returning generic messages in production</t>
+  </si>
+  <si>
+    <t>SCA-01</t>
+  </si>
+  <si>
+    <t>Dependency</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Supply Chain</t>
+  </si>
+  <si>
+    <t>proxy-addr</t>
+  </si>
+  <si>
+    <t>Updated to 2.0.8 (GHSA-jqcg-44mw-7w3h fixed)</t>
+  </si>
+  <si>
+    <t>SCA-02</t>
+  </si>
+  <si>
+    <t>shell-quote</t>
+  </si>
+  <si>
+    <t>Updated to 1.12.0 (GHSA-pqg4-j6r4-53mv fixed)</t>
+  </si>
+  <si>
+    <t>SCA-03</t>
+  </si>
+  <si>
+    <t>vite</t>
+  </si>
+  <si>
+    <t>Upgraded to 8.3.5 (GHSA-587h-7wmj-h5pm fixed)</t>
+  </si>
+  <si>
+    <t>SCA-04</t>
+  </si>
+  <si>
+    <t>body-parser</t>
+  </si>
+  <si>
+    <t>Updated to 2.4.0 (GHSA-27r3-jxmh-p828 fixed)</t>
+  </si>
+  <si>
+    <t>SCA-05</t>
+  </si>
+  <si>
+    <t>brace-expansion</t>
+  </si>
+  <si>
+    <t>Updated to 2.1.7 and 1.1.21</t>
+  </si>
+  <si>
+    <t>SCA-06</t>
+  </si>
+  <si>
+    <t>source-map-js</t>
+  </si>
+  <si>
+    <t>Updated to 1.2.2 (GHSA-68fv-2mgg-jv7q fixed)</t>
+  </si>
+  <si>
+    <t>SCA-07</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
+    <t>qs</t>
+  </si>
+  <si>
+    <t>Updated to 6.16.1 (GHSA-x5fp-wj9c-mxmx fixed)</t>
+  </si>
+  <si>
+    <t>SCA-08</t>
+  </si>
+  <si>
+    <t>@react-navigation/core</t>
+  </si>
+  <si>
+    <t>Updated to 7.24.0 (GHSA-vcc3-ghjq-m6fr fixed)</t>
+  </si>
+  <si>
+    <t>SCA-09</t>
+  </si>
+  <si>
+    <t>node-forge (@expo/cli)</t>
+  </si>
+  <si>
+    <t>Tied to Expo SDK 58; downgrade to Expo 44 would break React 19</t>
+  </si>
+  <si>
+    <t>SCA-10</t>
+  </si>
+  <si>
+    <t>zod (@expo/cli)</t>
+  </si>
+  <si>
+    <t>Tied to Expo SDK 58 config parser; downgrade to Expo 44 breaking</t>
+  </si>
+  <si>
+    <t>SCA-11</t>
+  </si>
+  <si>
+    <t>uuid (exceljs)</t>
+  </si>
+  <si>
+    <t>Downgrade to exceljs@3.4.0 is breaking; internal UUIDs only</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -218,8 +465,12 @@
       <b/>
       <color rgb="166534"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="92400E"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -246,6 +497,11 @@
         <fgColor rgb="DCFCE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -259,7 +515,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -269,6 +525,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -609,12 +866,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="3" width="20" customWidth="1"/>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -690,7 +948,7 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
@@ -703,89 +961,144 @@
       <c r="D9" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E9" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="6" t="s">
+      <c r="B10" s="5">
+        <v>2</v>
+      </c>
+      <c r="C10" s="5">
+        <v>2</v>
+      </c>
+      <c r="D10" s="5">
+        <v>0</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="B11" s="5">
+        <v>2</v>
+      </c>
+      <c r="C11" s="5">
+        <v>2</v>
+      </c>
+      <c r="D11" s="5">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="B12" s="5">
+        <v>2</v>
+      </c>
+      <c r="C12" s="5">
+        <v>2</v>
+      </c>
+      <c r="D12" s="5">
+        <v>0</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="5">
+        <v>2</v>
+      </c>
+      <c r="C13" s="5">
+        <v>2</v>
+      </c>
+      <c r="D13" s="5">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="5">
+        <v>9</v>
+      </c>
+      <c r="C14" s="5">
+        <v>4</v>
+      </c>
+      <c r="D14" s="5">
+        <v>5</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="B15" s="5">
+        <v>6</v>
+      </c>
+      <c r="C15" s="5">
+        <v>4</v>
+      </c>
+      <c r="D15" s="5">
+        <v>2</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="5">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5">
+        <v>0</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="5">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5">
+        <v>0</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -800,7 +1113,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -808,227 +1121,681 @@
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>32</v>
+      <c r="A1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>40</v>
       </c>
+      <c r="C4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>86</v>
+      </c>
       <c r="B4" s="5" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>41</v>
+        <v>87</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>43</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>43</v>
-      </c>
       <c r="F6" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>51</v>
+        <v>97</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>35</v>
+        <v>94</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>47</v>
+        <v>98</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>52</v>
+        <v>101</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>35</v>
+        <v>103</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>47</v>
+        <v>104</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>43</v>
+        <v>105</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>53</v>
+        <v>107</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>49</v>
+        <v>103</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>42</v>
+        <v>104</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>43</v>
+        <v>108</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>53</v>
+        <v>110</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>42</v>
+        <v>104</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>43</v>
+        <v>111</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>55</v>
+        <v>113</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>42</v>
+        <v>104</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>43</v>
+        <v>114</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>38</v>
+        <v>16</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(security): resolve dependency findings and document residual risks
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/Security_Review_Report.xlsx
+++ b/Vulnerability Test Results/Security_Review_Report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="144">
   <si>
     <t>CODESAGA APPLICATION - SAST SECURITY &amp; DEVSECOPS AUDIT REPORT</t>
   </si>
@@ -84,22 +84,22 @@
     <t>App Code — Low (PII Logging &amp; Error Leaks)</t>
   </si>
   <si>
-    <t>Dependencies (SCA) — Critical (proxy-addr, shell-quote)</t>
+    <t>Dependencies (SCA) — Critical (proxy-addr, shell-quote, form-data)</t>
   </si>
   <si>
     <t>REMEDIATED (0 Critical Remaining)</t>
   </si>
   <si>
-    <t>Dependencies (SCA) — High (Vite, body-parser, brace-expansion)</t>
-  </si>
-  <si>
-    <t>PARTIALLY REMEDIATED (5 in Expo CLI)</t>
+    <t>Dependencies (SCA) — High (Vite, body-parser, brace-expansion, source-map, serialize-js)</t>
+  </si>
+  <si>
+    <t>PARTIALLY REMEDIATED (2 in Expo CLI)</t>
   </si>
   <si>
     <t>Dependencies (SCA) — Moderate (qs, query-string, uuid)</t>
   </si>
   <si>
-    <t>PARTIALLY REMEDIATED (2 in exceljs/uuid)</t>
+    <t>REMEDIATED (0 Moderate Remaining)</t>
   </si>
   <si>
     <t>Hardcoded Secrets (Gitleaks)</t>
@@ -408,7 +408,7 @@
     <t>node-forge (@expo/cli)</t>
   </si>
   <si>
-    <t>Tied to Expo SDK 58; downgrade to Expo 44 would break React 19</t>
+    <t>Tied to Expo SDK 58 dev cert generation; no patched release exists on npm</t>
   </si>
   <si>
     <t>SCA-10</t>
@@ -417,7 +417,7 @@
     <t>zod (@expo/cli)</t>
   </si>
   <si>
-    <t>Tied to Expo SDK 58 config parser; downgrade to Expo 44 breaking</t>
+    <t>Tied to Expo SDK 58 config parser; Zod 4 upgrade is breaking</t>
   </si>
   <si>
     <t>SCA-11</t>
@@ -426,7 +426,25 @@
     <t>uuid (exceljs)</t>
   </si>
   <si>
-    <t>Downgrade to exceljs@3.4.0 is breaking; internal UUIDs only</t>
+    <t>Resolved via safe override to uuid@^11.1.1 across root and test workspaces</t>
+  </si>
+  <si>
+    <t>SCA-12</t>
+  </si>
+  <si>
+    <t>serialize-javascript (mocha)</t>
+  </si>
+  <si>
+    <t>Resolved via selenium-tests override to serialize-javascript@^7.1.4</t>
+  </si>
+  <si>
+    <t>SCA-13</t>
+  </si>
+  <si>
+    <t>form-data (appium)</t>
+  </si>
+  <si>
+    <t>Resolved via appium-tests override to form-data@^4.0.6 (GHSA-fjxv-7rqg-78g4 fixed)</t>
   </si>
 </sst>
 </file>
@@ -1021,10 +1039,10 @@
         <v>23</v>
       </c>
       <c r="B13" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" s="5">
         <v>0</v>
@@ -1041,10 +1059,10 @@
         <v>9</v>
       </c>
       <c r="C14" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D14" s="5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>26</v>
@@ -1055,15 +1073,15 @@
         <v>27</v>
       </c>
       <c r="B15" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C15" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" s="5">
-        <v>2</v>
-      </c>
-      <c r="E15" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1372,7 +1390,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1791,11 +1809,57 @@
       <c r="E18" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>17</v>
+      <c r="F18" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>137</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(ci): resolve selenium dom locators, configure api baseline scope, add sec-02 auth stress suite, and bundle 4 reports
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/Security_Review_Report.xlsx
+++ b/Vulnerability Test Results/Security_Review_Report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="148">
   <si>
     <t>CODESAGA APPLICATION - SAST SECURITY &amp; DEVSECOPS AUDIT REPORT</t>
   </si>
@@ -27,7 +27,7 @@
     <t>Audit Date:</t>
   </si>
   <si>
-    <t>26/10/2026</t>
+    <t>28/10/2026</t>
   </si>
   <si>
     <t>Technology Stack:</t>
@@ -45,13 +45,13 @@
     <t>Target Scope:</t>
   </si>
   <si>
-    <t>Backend API, Authentication, Models, Routes</t>
+    <t>Backend API, Authentication, Models, Dependencies</t>
   </si>
   <si>
     <t>Remediation Status:</t>
   </si>
   <si>
-    <t>Remediated &amp; Verified (20/20 Tests Passed)</t>
+    <t>Partially Remediated (17/19 Fixed, 2 Documented Pending in Expo CLI)</t>
   </si>
   <si>
     <t>🛡️ RECONCILED SECURITY FINDINGS &amp; REMEDIATION METRICS</t>
@@ -72,16 +72,16 @@
     <t>Verification Status</t>
   </si>
   <si>
-    <t>App Code — High (IDOR &amp; Rate Limiting)</t>
+    <t>Application Code — High (SEC-01 IDOR, SEC-02 Rate Limiting)</t>
   </si>
   <si>
     <t>REMEDIATED (Verified via Tests)</t>
   </si>
   <si>
-    <t>App Code — Medium (Headers &amp; Validation)</t>
-  </si>
-  <si>
-    <t>App Code — Low (PII Logging &amp; Error Leaks)</t>
+    <t>Application Code — Medium (SEC-03 Headers, SEC-04 Input Validation)</t>
+  </si>
+  <si>
+    <t>Application Code — Low (SEC-05 PII Masking, SEC-06 Error Sanitization)</t>
   </si>
   <si>
     <t>Dependencies (SCA) — Critical (proxy-addr, shell-quote, form-data)</t>
@@ -90,10 +90,16 @@
     <t>REMEDIATED (0 Critical Remaining)</t>
   </si>
   <si>
-    <t>Dependencies (SCA) — High (Vite, body-parser, brace-expansion, source-map, serialize-js)</t>
-  </si>
-  <si>
-    <t>PARTIALLY REMEDIATED (2 in Expo CLI)</t>
+    <t>Dependencies (SCA) — High Remediated (Vite, body-parser, brace-expansion, source-map, serialize-js)</t>
+  </si>
+  <si>
+    <t>REMEDIATED (5 Highs Patched)</t>
+  </si>
+  <si>
+    <t>Dependencies (SCA) — High Documented Pending (node-forge, zod in @expo/cli)</t>
+  </si>
+  <si>
+    <t>DOCUMENTED PENDING (Retained: Breaking in Expo SDK 58)</t>
   </si>
   <si>
     <t>Dependencies (SCA) — Moderate (qs, query-string, uuid)</t>
@@ -106,6 +112,12 @@
   </si>
   <si>
     <t>CLEAN (0 Secrets Detected)</t>
+  </si>
+  <si>
+    <t>Total Findings Register (findings.csv)</t>
+  </si>
+  <si>
+    <t>PARTIALLY REMEDIATED (17/19 Remediated, 2 Documented Pending)</t>
   </si>
   <si>
     <t>Critical Security Gate Policy</t>
@@ -884,13 +896,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="1" max="1" width="80" customWidth="1"/>
     <col min="2" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="34" customWidth="1"/>
+    <col min="5" max="5" width="45" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1056,15 +1068,15 @@
         <v>25</v>
       </c>
       <c r="B14" s="5">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C14" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D14" s="5">
-        <v>2</v>
-      </c>
-      <c r="E14" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1073,15 +1085,15 @@
         <v>27</v>
       </c>
       <c r="B15" s="5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C15" s="5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D15" s="5">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1090,10 +1102,10 @@
         <v>29</v>
       </c>
       <c r="B16" s="5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C16" s="5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D16" s="5">
         <v>0</v>
@@ -1117,6 +1129,40 @@
       </c>
       <c r="E17" s="6" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="5">
+        <v>19</v>
+      </c>
+      <c r="C18" s="5">
+        <v>17</v>
+      </c>
+      <c r="D18" s="5">
+        <v>2</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="5">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5">
+        <v>0</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1144,242 +1190,242 @@
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>41</v>
-      </c>
       <c r="D3" s="5" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>49</v>
-      </c>
       <c r="F5" s="6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>52</v>
-      </c>
       <c r="C6" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="E11" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="E12" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1404,462 +1450,462 @@
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>79</v>
-      </c>
       <c r="C3" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>103</v>
-      </c>
       <c r="D9" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>17</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>17</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ci): run eight 500-case suites with master Excel and verified ownership auth
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/Security_Review_Report.xlsx
+++ b/Vulnerability Test Results/Security_Review_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="211">
   <si>
     <t>CodeSaga security evidence</t>
   </si>
@@ -22,13 +22,13 @@
     <t>Base commit (local working tree snapshot)</t>
   </si>
   <si>
-    <t>197b8541391733c620052ddcc9f8aef3e8315de3</t>
+    <t>4582dff01e117cf0d7e8bff54e79b46aa9a1aa87</t>
   </si>
   <si>
     <t>Generated UTC</t>
   </si>
   <si>
-    <t>2026-10-28T08:40:31.806Z</t>
+    <t>2026-10-28T09:26:58.601Z</t>
   </si>
   <si>
     <t>Register scope</t>
@@ -91,7 +91,7 @@
     <t>Release status</t>
   </si>
   <si>
-    <t>BLOCKED: reopened SEC-01 authentication issue; incomplete mobile coverage; residual Low dependency findings.</t>
+    <t>Source authentication fix tested. Verify production deployment/email configuration separately; residual Low dependencies remain.</t>
   </si>
   <si>
     <t>Counts</t>
@@ -145,10 +145,10 @@
     <t>Insecure Direct Object Reference (IDOR / BOLA) via email route parameter</t>
   </si>
   <si>
-    <t>Pending</t>
-  </si>
-  <si>
-    <t>REOPENED: protected resource routes check HMAC ownership but POST /api/users/login issues tokens from email alone; registration can overwrite existing passwords and set-password lacks server-verified ownership proof. Require authenticated ownership or a server-verified single-use OTP grant before token issuance or credential changes. Production-router negative tests remain required.</t>
+    <t>Remediated</t>
+  </si>
+  <si>
+    <t>Closed in source: login registration and password changes require own signed session or server-verified single-use email ownership grant; public lookup redacts account progress/certificates. Server CSPRNG OTP has expiry attempt limits email binding and replay protection. Actual-router ownership regression and 500 attack-denial cases verify the fix. Production deployment/email configuration requires separate verification.</t>
   </si>
   <si>
     <t>SEC-02</t>
@@ -163,9 +163,6 @@
     <t>Absence of rate limiting allows credential brute-force and CPU exhaustion via bcrypt</t>
   </si>
   <si>
-    <t>Remediated</t>
-  </si>
-  <si>
     <t>Integrated sliding-window IP rate limiter authRateLimiter (10 attempts per 15 min with HTTP 429 and Retry-After header)</t>
   </si>
   <si>
@@ -496,39 +493,42 @@
     <t>POST</t>
   </si>
   <si>
-    <t>No (Self-Registration)</t>
+    <t>Verified email ownership grant</t>
+  </si>
+  <si>
+    <t>Email owner</t>
+  </si>
+  <si>
+    <t>Register new detective user account</t>
+  </si>
+  <si>
+    <t>Requires own signed session or single-use server-verified email grant; normalizes email; password complexity validation (8+ chars letter+number); bcrypt 12 rounds; returns HMAC auth token</t>
+  </si>
+  <si>
+    <t>/api/users/set-password</t>
+  </si>
+  <si>
+    <t>Own session or verified email grant</t>
+  </si>
+  <si>
+    <t>Account owner</t>
+  </si>
+  <si>
+    <t>Configure or change account password</t>
+  </si>
+  <si>
+    <t>Own signed session or server-verified single-use grant; rate limited (10 attempts per 15 min); password complexity check; bcrypt 12 rounds; returns HMAC auth token</t>
+  </si>
+  <si>
+    <t>/api/users/login-password</t>
+  </si>
+  <si>
+    <t>Password credentials (Rate-Limited)</t>
   </si>
   <si>
     <t>Public / User</t>
   </si>
   <si>
-    <t>Register new detective user account</t>
-  </si>
-  <si>
-    <t>SEC-01 PENDING: existing account password overwrite; normalizes email; password complexity validation (8+ chars letter+number); bcrypt 12 rounds; returns HMAC auth token</t>
-  </si>
-  <si>
-    <t>/api/users/set-password</t>
-  </si>
-  <si>
-    <t>No ownership proof (Rate-Limited)</t>
-  </si>
-  <si>
-    <t>Unverified caller</t>
-  </si>
-  <si>
-    <t>Configure or change account password</t>
-  </si>
-  <si>
-    <t>SEC-01 PENDING: no ownership proof; rate limited (10 attempts per 15 min); password complexity check; bcrypt 12 rounds; returns HMAC auth token</t>
-  </si>
-  <si>
-    <t>/api/users/login-password</t>
-  </si>
-  <si>
-    <t>Password credentials (Rate-Limited)</t>
-  </si>
-  <si>
     <t>Authenticate existing account with email + password</t>
   </si>
   <si>
@@ -541,7 +541,7 @@
     <t>Record user login timestamp</t>
   </si>
   <si>
-    <t>SEC-01 PENDING: email-only token issuance; updates lastLogin date in MongoDB Atlas; deletes password_hash from response; returns HMAC auth token</t>
+    <t>Signed ownership or verified email grant required; updates lastLogin date in MongoDB Atlas; deletes password_hash from response; returns HMAC auth token</t>
   </si>
   <si>
     <t>/api/users/:email/progress</t>
@@ -647,18 +647,6 @@
   </si>
   <si>
     <t>&gt;=52.0.0-canary-20240625-2333e70</t>
-  </si>
-  <si>
-    <t>diff</t>
-  </si>
-  <si>
-    <t>6.0.0 - 8.0.2</t>
-  </si>
-  <si>
-    <t>mocha</t>
-  </si>
-  <si>
-    <t>11.4.0 - 12.0.0-beta-3</t>
   </si>
 </sst>
 </file>
@@ -1104,10 +1092,10 @@
         <v>6</v>
       </c>
       <c r="C6" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1132,10 +1120,10 @@
         <v>19</v>
       </c>
       <c r="C8" s="3">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1192,10 +1180,10 @@
         <v>0</v>
       </c>
       <c r="E12" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F12" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1246,7 +1234,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" ht="70" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="84" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
@@ -1307,7 +1295,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" ht="126" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="140" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>37</v>
       </c>
@@ -1359,73 +1347,73 @@
         <v>48</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="4" ht="56" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="5" ht="56" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>40</v>
       </c>
       <c r="F5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>38</v>
@@ -1434,27 +1422,27 @@
         <v>16</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="7" ht="56" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>38</v>
@@ -1463,399 +1451,399 @@
         <v>16</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>71</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>73</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>74</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E9" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E10" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>88</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>76</v>
-      </c>
       <c r="F11" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F12" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G12" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="H12" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I12" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F13" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H13" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I13" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>76</v>
-      </c>
       <c r="F14" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="H15" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I15" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="16" ht="70" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E16" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I16" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="17" ht="70" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G17" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="H17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I17" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E18" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="H18" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I18" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E19" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="H19" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I19" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="20" ht="56" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E20" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="G20" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="H20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I20" s="3" t="s">
         <v>133</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1876,157 +1864,157 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>147</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>150</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="G4" s="3" t="s">
+    </row>
+    <row r="5" ht="70" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="5" ht="56" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>162</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="6" ht="56" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>167</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>161</v>
-      </c>
       <c r="E7" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>171</v>
@@ -2040,16 +2028,16 @@
         <v>173</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>174</v>
@@ -2063,7 +2051,7 @@
         <v>176</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>177</v>
@@ -2072,7 +2060,7 @@
         <v>178</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>179</v>
@@ -2095,7 +2083,7 @@
         <v>178</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>182</v>
@@ -2109,7 +2097,7 @@
         <v>184</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>177</v>
@@ -2118,7 +2106,7 @@
         <v>178</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>185</v>
@@ -2141,7 +2129,7 @@
         <v>178</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>187</v>
@@ -2158,7 +2146,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2326,46 +2314,6 @@
         <v>201</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>198</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>